<commit_message>
open pages bug fixed && download flow merge
</commit_message>
<xml_diff>
--- a/Data/08 25 CONTROL TRABAJADOR INDEPENDIENTE AGOSTO 2025.xlsx
+++ b/Data/08 25 CONTROL TRABAJADOR INDEPENDIENTE AGOSTO 2025.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-05-20 13:31:07</t>
+          <t>2026-06-03 11:57:17</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>C:\Users\Dembe\Proyects\Python\AsistenteIMSS\Data\08 MENSAJE TI AGOSTO TOTAL id.pdf</t>
+          <t>C:\Users\Dembe\Proyects\Python\AsistenteIMSS\Data\pdf\ALBERTO FLORES AVILA\Comprobante.pdf</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: actualiza archivos de pruebas y documentación
</commit_message>
<xml_diff>
--- a/Data/08 25 CONTROL TRABAJADOR INDEPENDIENTE AGOSTO 2025.xlsx
+++ b/Data/08 25 CONTROL TRABAJADOR INDEPENDIENTE AGOSTO 2025.xlsx
@@ -695,7 +695,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-06-11 12:10:20</t>
+          <t>2026-07-21 14:05:09</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>C:\Users\Dembe\Proyects\Python\AsistenteIMSS\Data\pdf\ALBERTO FLORES AVILA\Comprobante.pdf</t>
+          <t>C:\Users\sofia\Proyects\IMSS\prueba_imss\prueba_indep\ALBERTO FLORES AVILA\Comprobante (1).pdf</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr"/>
@@ -721,7 +721,7 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>C:/Users/Dembe/Proyects/Python/AsistenteIMSS/Data/pdf</t>
+          <t>C:/Users/sofia/Proyects/IMSS/prueba_imss/prueba_indep</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr"/>
@@ -810,7 +810,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>2026-05-17 22:46:41</t>
+          <t>2026-07-21 14:07:03</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -820,7 +820,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>C:\Users\Dembe\Proyects\Python\AsistenteIMSS\Data\pdf\ALDO JOSUE COVA GONZALEZ\Comprobante.pdf</t>
+          <t>C:\Users\sofia\Proyects\IMSS\prueba_imss\prueba_indep\ALDO JOSUE COVA GONZALEZ\Comprobante.pdf</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr"/>
@@ -836,7 +836,7 @@
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>C:/Users/Dembe/Proyects/Python/AsistenteIMSS/Data/pdf</t>
+          <t>C:/Users/sofia/Proyects/IMSS/prueba_imss/prueba_indep</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr"/>

</xml_diff>